<commit_message>
added new function in utl to process html content for upmc payer
</commit_message>
<xml_diff>
--- a/errors.xlsx
+++ b/errors.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29523"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{2C3F3EFF-A5B2-4EFF-BDCF-C666A2066436}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{D2364AB6-F01D-4CBD-A3FB-3D7B997EF23E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="32">
   <si>
     <t>Company Name</t>
   </si>
@@ -75,31 +75,58 @@
     <t>Source Link</t>
   </si>
   <si>
-    <t>Cigna</t>
-  </si>
-  <si>
-    <t>Cigna TotalCare (HMO D-SNP)</t>
-  </si>
-  <si>
-    <t>Alabama</t>
-  </si>
-  <si>
-    <t>https://www.cigna.com/static/www-cigna-com/docs/medicare/plans-services/2025/formulary-saver.pdf</t>
-  </si>
-  <si>
-    <t>1-855-278-5614</t>
-  </si>
-  <si>
-    <t>11501 Alterra Parkway</t>
-  </si>
-  <si>
-    <t>Suite 500</t>
-  </si>
-  <si>
-    <t>Austin</t>
-  </si>
-  <si>
-    <t>https://plans.cigna.com/plan-details?zip=35203&amp;fip=01073&amp;PlanType=MAPD&amp;PlanID=1N1VDL7WCS&amp;PlanYear=2025&amp;previousAnchor=ma#plandocuments</t>
+    <t>BCBS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BCN HRASM PCP Focus -Individual and family </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Michigan </t>
+  </si>
+  <si>
+    <t>https://www.bcbsm.com/amslibs/content/dam/public/marketplace/2025-individual/documents/custom-select-drug-list/six-tier.pdf</t>
+  </si>
+  <si>
+    <t>1-888-288-2738</t>
+  </si>
+  <si>
+    <t>600 E. Lafayette Blvd.</t>
+  </si>
+  <si>
+    <t>Detroit</t>
+  </si>
+  <si>
+    <t>Michigan</t>
+  </si>
+  <si>
+    <t>https://www.bcbsm.com/individuals/resources/forms-documents/drug-lists/2025-drug-lists/</t>
+  </si>
+  <si>
+    <t>Medicare Plus BlueSM PPO Part B Credit</t>
+  </si>
+  <si>
+    <t>https://www.bcbsm.com/amslibs/content/dam/microsites/medicare/documents/2025/pharmacy/formulary-ppo-essential-meijer-part-b.pdf</t>
+  </si>
+  <si>
+    <t>https://www.bcbsm.com/medicare/resources/forms-documents/drug-lists-2025/</t>
+  </si>
+  <si>
+    <t>Group BCN Advantage HMO and HMO-POS</t>
+  </si>
+  <si>
+    <t>https://www.bcbsm.com/amslibs/content/dam/microsites/medicare/documents/2025/pharmacy/formulary-bcna-group.pdf</t>
+  </si>
+  <si>
+    <t>Blue Cross Metro Detroit HMO-Large,Small Group</t>
+  </si>
+  <si>
+    <t>https://www.bcbsm.com/individuals/resources/forms-documents/drug-lists/group/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Blue Cross Blue Shield of Michigan and Blue Care Network Preferred Drug List </t>
+  </si>
+  <si>
+    <t>https://www.bcbsm.com/amslibs/content/dam/public/consumer/forms-documents/pharmacy/preferred-drug-list.pdf</t>
   </si>
 </sst>
 </file>
@@ -182,7 +209,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -194,6 +221,9 @@
     <xf numFmtId="14" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -529,7 +559,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:N2"/>
+  <dimension ref="A1:N6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="26.28515625" bestFit="1" customWidth="1"/>
@@ -593,51 +623,217 @@
       </c>
     </row>
     <row r="2" spans="1:14" ht="15.75">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="D2" s="2"/>
-      <c r="E2" s="3" t="s">
+      <c r="D2" s="5"/>
+      <c r="E2" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="F2" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="G2" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="H2" s="2" t="s">
+      <c r="H2" s="5"/>
+      <c r="I2" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="I2" s="2" t="s">
+      <c r="J2" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="J2" s="2" t="s">
+      <c r="K2" s="5">
+        <v>48226</v>
+      </c>
+      <c r="L2" s="7">
+        <v>45931</v>
+      </c>
+      <c r="M2" s="7">
+        <v>45947</v>
+      </c>
+      <c r="N2" s="6" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" ht="15.75">
+      <c r="A3" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C3" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="K2" s="2">
-        <v>78758</v>
-      </c>
-      <c r="L2" s="4">
+      <c r="D3" s="2"/>
+      <c r="E3" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="H3" s="2"/>
+      <c r="I3" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="J3" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="K3" s="2">
+        <v>48226</v>
+      </c>
+      <c r="L3" s="4">
         <v>45931</v>
       </c>
-      <c r="M2" s="4">
-        <v>45940</v>
-      </c>
-      <c r="N2" s="3" t="s">
-        <v>22</v>
+      <c r="M3" s="4">
+        <v>45947</v>
+      </c>
+      <c r="N3" s="3" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" ht="15.75">
+      <c r="A4" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="D4" s="2"/>
+      <c r="E4" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="H4" s="2"/>
+      <c r="I4" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="J4" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="K4" s="2">
+        <v>48226</v>
+      </c>
+      <c r="L4" s="4">
+        <v>45931</v>
+      </c>
+      <c r="M4" s="4">
+        <v>45947</v>
+      </c>
+      <c r="N4" s="3" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" ht="15.75">
+      <c r="A5" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="D5" s="2"/>
+      <c r="E5" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="H5" s="2"/>
+      <c r="I5" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="J5" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="K5" s="2">
+        <v>48226</v>
+      </c>
+      <c r="L5" s="4">
+        <v>45931</v>
+      </c>
+      <c r="M5" s="4">
+        <v>45947</v>
+      </c>
+      <c r="N5" s="3" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" ht="15.75">
+      <c r="A6" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="D6" s="2"/>
+      <c r="E6" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="H6" s="2"/>
+      <c r="I6" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="J6" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="K6" s="2">
+        <v>48226</v>
+      </c>
+      <c r="L6" s="4">
+        <v>45931</v>
+      </c>
+      <c r="M6" s="4">
+        <v>45947</v>
+      </c>
+      <c r="N6" s="3" t="s">
+        <v>29</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="E2" r:id="rId1" xr:uid="{BC658594-5F20-4E54-B3B8-B2A0DF68BA3D}"/>
-    <hyperlink ref="N2" r:id="rId2" location="plandocuments" xr:uid="{CCF656F8-A6F1-4509-8152-D10E42484956}"/>
+    <hyperlink ref="E2" r:id="rId1" xr:uid="{7DF4D1CA-FF22-473D-B2F2-0CD6676FE09A}"/>
+    <hyperlink ref="N2" r:id="rId2" xr:uid="{5D120FAB-99E4-41CC-B47E-3039C0013CC7}"/>
+    <hyperlink ref="E3" r:id="rId3" xr:uid="{F2ACE8F4-D888-4D8D-BC17-D4D669EC1EC0}"/>
+    <hyperlink ref="N3" r:id="rId4" xr:uid="{50D2A0A6-B2F3-4FA7-AA92-3D3218D547C5}"/>
+    <hyperlink ref="E4" r:id="rId5" xr:uid="{470F50E6-C2FA-48AC-B31A-D9E36DC1FCE3}"/>
+    <hyperlink ref="N4" r:id="rId6" xr:uid="{575E08D9-F708-42D4-A434-E4ACC27FFE07}"/>
+    <hyperlink ref="E5" r:id="rId7" xr:uid="{BE87AE35-7FA1-4CDB-84FF-E829BB9C26DE}"/>
+    <hyperlink ref="N5" r:id="rId8" xr:uid="{AA8FF877-8433-4E7F-AFA0-8576ACE92E7F}"/>
+    <hyperlink ref="E6" r:id="rId9" xr:uid="{E780ED64-96C5-4812-AECB-70DC6FE4F67B}"/>
+    <hyperlink ref="N6" r:id="rId10" xr:uid="{C5297EFA-B336-4E5C-86C8-1A49D49DC512}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
added range page numbers, enhance pdf function, mg issue handling
</commit_message>
<xml_diff>
--- a/errors.xlsx
+++ b/errors.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29523"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29607"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D2364AB6-F01D-4CBD-A3FB-3D7B997EF23E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{45807574-AB1B-4D95-BA83-AC093D32F0A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="23">
   <si>
     <t>Company Name</t>
   </si>
@@ -42,9 +42,6 @@
     <t>States Covered</t>
   </si>
   <si>
-    <t>County</t>
-  </si>
-  <si>
     <t>Formulary URL</t>
   </si>
   <si>
@@ -75,65 +72,41 @@
     <t>Source Link</t>
   </si>
   <si>
-    <t>BCBS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BCN HRASM PCP Focus -Individual and family </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Michigan </t>
-  </si>
-  <si>
-    <t>https://www.bcbsm.com/amslibs/content/dam/public/marketplace/2025-individual/documents/custom-select-drug-list/six-tier.pdf</t>
-  </si>
-  <si>
-    <t>1-888-288-2738</t>
-  </si>
-  <si>
-    <t>600 E. Lafayette Blvd.</t>
-  </si>
-  <si>
-    <t>Detroit</t>
-  </si>
-  <si>
-    <t>Michigan</t>
-  </si>
-  <si>
-    <t>https://www.bcbsm.com/individuals/resources/forms-documents/drug-lists/2025-drug-lists/</t>
-  </si>
-  <si>
-    <t>Medicare Plus BlueSM PPO Part B Credit</t>
-  </si>
-  <si>
-    <t>https://www.bcbsm.com/amslibs/content/dam/microsites/medicare/documents/2025/pharmacy/formulary-ppo-essential-meijer-part-b.pdf</t>
-  </si>
-  <si>
-    <t>https://www.bcbsm.com/medicare/resources/forms-documents/drug-lists-2025/</t>
-  </si>
-  <si>
-    <t>Group BCN Advantage HMO and HMO-POS</t>
-  </si>
-  <si>
-    <t>https://www.bcbsm.com/amslibs/content/dam/microsites/medicare/documents/2025/pharmacy/formulary-bcna-group.pdf</t>
-  </si>
-  <si>
-    <t>Blue Cross Metro Detroit HMO-Large,Small Group</t>
-  </si>
-  <si>
-    <t>https://www.bcbsm.com/individuals/resources/forms-documents/drug-lists/group/</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Blue Cross Blue Shield of Michigan and Blue Care Network Preferred Drug List </t>
-  </si>
-  <si>
-    <t>https://www.bcbsm.com/amslibs/content/dam/public/consumer/forms-documents/pharmacy/preferred-drug-list.pdf</t>
+    <t>Zing health</t>
+  </si>
+  <si>
+    <t>H4624-012 Zing Select Diabetes &amp; Heart MI (HMO C-SNP)</t>
+  </si>
+  <si>
+    <t>Illinois</t>
+  </si>
+  <si>
+    <t>https://www.myzinghealth.com/uploads/member_option/2025_Zing_CSNP_ENG_Comp_Formulary.pdf</t>
+  </si>
+  <si>
+    <t>1-866-946-4458</t>
+  </si>
+  <si>
+    <t>225 W. Washington St</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Suite 450 </t>
+  </si>
+  <si>
+    <t>Chicago</t>
+  </si>
+  <si>
+    <t>https://www.myzinghealth.com/pharmacy/covered_drugs</t>
+  </si>
+  <si>
+    <t>Simyrna</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -148,11 +121,6 @@
       <name val="Times New Roman"/>
     </font>
     <font>
-      <sz val="12"/>
-      <color rgb="FF000000"/>
-      <name val="Times New Roman"/>
-    </font>
-    <font>
       <u/>
       <sz val="11"/>
       <color theme="10"/>
@@ -161,10 +129,22 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <u/>
-      <sz val="12"/>
-      <color theme="10"/>
-      <name val="Times New Roman"/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF242424"/>
+      <name val="Aptos Narrow"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="3">
@@ -207,23 +187,20 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="14" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="14" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -559,26 +536,28 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:N6"/>
+  <dimension ref="A1:O2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="26.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="30.28515625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="82.7109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="16" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8.42578125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="194.28515625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="16.7109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="33.28515625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="32.7109375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="12.7109375" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="14.28515625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="6.85546875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="16.7109375" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="15.85546875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="103.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="194.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="23.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="33.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="32.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="14.140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="16.7109375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="15.85546875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="103.28515625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="36.5703125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="10" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="21" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="15.75">
+    <row r="1" spans="1:15" ht="15.75">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -618,223 +597,52 @@
       <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+    </row>
+    <row r="2" spans="1:15" ht="29.25">
+      <c r="A2" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="2" spans="1:14" ht="15.75">
-      <c r="A2" s="5" t="s">
+      <c r="B2" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="C2" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="C2" s="5" t="s">
+      <c r="D2" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="D2" s="5"/>
-      <c r="E2" s="6" t="s">
+      <c r="E2" t="s">
         <v>17</v>
       </c>
-      <c r="F2" s="5" t="s">
+      <c r="F2" t="s">
         <v>18</v>
       </c>
-      <c r="G2" s="5" t="s">
+      <c r="G2" t="s">
         <v>19</v>
       </c>
-      <c r="H2" s="5"/>
-      <c r="I2" s="5" t="s">
+      <c r="H2" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="J2" s="5" t="s">
+      <c r="I2" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="J2" s="4">
+        <v>60606</v>
+      </c>
+      <c r="K2" s="2">
+        <v>45962</v>
+      </c>
+      <c r="L2" s="2">
+        <v>45975</v>
+      </c>
+      <c r="N2" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="K2" s="5">
-        <v>48226</v>
-      </c>
-      <c r="L2" s="7">
-        <v>45931</v>
-      </c>
-      <c r="M2" s="7">
-        <v>45947</v>
-      </c>
-      <c r="N2" s="6" t="s">
+      <c r="O2" t="s">
         <v>22</v>
-      </c>
-    </row>
-    <row r="3" spans="1:14" ht="15.75">
-      <c r="A3" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="D3" s="2"/>
-      <c r="E3" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="G3" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="H3" s="2"/>
-      <c r="I3" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="J3" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="K3" s="2">
-        <v>48226</v>
-      </c>
-      <c r="L3" s="4">
-        <v>45931</v>
-      </c>
-      <c r="M3" s="4">
-        <v>45947</v>
-      </c>
-      <c r="N3" s="3" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="4" spans="1:14" ht="15.75">
-      <c r="A4" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="D4" s="2"/>
-      <c r="E4" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="F4" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="G4" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="H4" s="2"/>
-      <c r="I4" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="J4" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="K4" s="2">
-        <v>48226</v>
-      </c>
-      <c r="L4" s="4">
-        <v>45931</v>
-      </c>
-      <c r="M4" s="4">
-        <v>45947</v>
-      </c>
-      <c r="N4" s="3" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="5" spans="1:14" ht="15.75">
-      <c r="A5" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="D5" s="2"/>
-      <c r="E5" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="F5" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="G5" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="H5" s="2"/>
-      <c r="I5" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="J5" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="K5" s="2">
-        <v>48226</v>
-      </c>
-      <c r="L5" s="4">
-        <v>45931</v>
-      </c>
-      <c r="M5" s="4">
-        <v>45947</v>
-      </c>
-      <c r="N5" s="3" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="6" spans="1:14" ht="15.75">
-      <c r="A6" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="D6" s="2"/>
-      <c r="E6" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="F6" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="G6" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="H6" s="2"/>
-      <c r="I6" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="J6" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="K6" s="2">
-        <v>48226</v>
-      </c>
-      <c r="L6" s="4">
-        <v>45931</v>
-      </c>
-      <c r="M6" s="4">
-        <v>45947</v>
-      </c>
-      <c r="N6" s="3" t="s">
-        <v>29</v>
       </c>
     </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="E2" r:id="rId1" xr:uid="{7DF4D1CA-FF22-473D-B2F2-0CD6676FE09A}"/>
-    <hyperlink ref="N2" r:id="rId2" xr:uid="{5D120FAB-99E4-41CC-B47E-3039C0013CC7}"/>
-    <hyperlink ref="E3" r:id="rId3" xr:uid="{F2ACE8F4-D888-4D8D-BC17-D4D669EC1EC0}"/>
-    <hyperlink ref="N3" r:id="rId4" xr:uid="{50D2A0A6-B2F3-4FA7-AA92-3D3218D547C5}"/>
-    <hyperlink ref="E4" r:id="rId5" xr:uid="{470F50E6-C2FA-48AC-B31A-D9E36DC1FCE3}"/>
-    <hyperlink ref="N4" r:id="rId6" xr:uid="{575E08D9-F708-42D4-A434-E4ACC27FFE07}"/>
-    <hyperlink ref="E5" r:id="rId7" xr:uid="{BE87AE35-7FA1-4CDB-84FF-E829BB9C26DE}"/>
-    <hyperlink ref="N5" r:id="rId8" xr:uid="{AA8FF877-8433-4E7F-AFA0-8576ACE92E7F}"/>
-    <hyperlink ref="E6" r:id="rId9" xr:uid="{E780ED64-96C5-4812-AECB-70DC6FE4F67B}"/>
-    <hyperlink ref="N6" r:id="rId10" xr:uid="{C5297EFA-B336-4E5C-86C8-1A49D49DC512}"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
changed the code formatting and solved the index page issues
</commit_message>
<xml_diff>
--- a/errors.xlsx
+++ b/errors.xlsx
@@ -1,47 +1,104 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <workbookPr codeName="ThisWorkbook"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet sheetId="1" name="Sheet1" state="visible" r:id="rId4"/>
   </sheets>
+  <calcPr calcId="171027"/>
 </workbook>
 </file>
 
-<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
-  <metadataTypes count="1">
-    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
-  </metadataTypes>
-  <futureMetadata name="XLDAPR" count="1">
-    <bk>
-      <extLst>
-        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
-          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
-        </ext>
-      </extLst>
-    </bk>
-  </futureMetadata>
-  <cellMetadata count="1">
-    <bk>
-      <rc t="1" v="0"/>
-    </bk>
-  </cellMetadata>
-</metadata>
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
+  <si>
+    <t>Company Name</t>
+  </si>
+  <si>
+    <t>Plan Name</t>
+  </si>
+  <si>
+    <t>States Covered</t>
+  </si>
+  <si>
+    <t>Formulary URL</t>
+  </si>
+  <si>
+    <t>Contact Phone</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Communication Address Line 1 </t>
+  </si>
+  <si>
+    <t>Communication Address Line 2</t>
+  </si>
+  <si>
+    <t>City</t>
+  </si>
+  <si>
+    <t>State</t>
+  </si>
+  <si>
+    <t>Zip</t>
+  </si>
+  <si>
+    <t>Formulory date</t>
+  </si>
+  <si>
+    <t>Captured Date</t>
+  </si>
+  <si>
+    <t>Source Link</t>
+  </si>
+  <si>
+    <t>Hennepin Health</t>
+  </si>
+  <si>
+    <t>Hennepin Health-MNCare</t>
+  </si>
+  <si>
+    <t>https://cbg.adaptiverx.com/web/pdf?key=8F02B26A288102C27BAC82D14C006C6FC54D480F80409B6872E9A8AAA274F8DE</t>
+  </si>
+  <si>
+    <t>1-612-596-1036 (TTY 711)</t>
+  </si>
+  <si>
+    <t>300 South Sixth Street, MC 604</t>
+  </si>
+  <si>
+    <t>Minneapolis</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Minnesota</t>
+  </si>
+  <si>
+    <t>55487-0604</t>
+  </si>
+  <si>
+    <t>11/1/2025</t>
+  </si>
+  <si>
+    <t>11/14/2025</t>
+  </si>
+  <si>
+    <t>https://www.hennepinhealth.org/</t>
+  </si>
+  <si>
+    <t>Madhan</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <numFmts count="1">
-    <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
-  </numFmts>
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
-      <sz val="12"/>
       <color theme="1"/>
-      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="2">
@@ -65,13 +122,21 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -396,103 +461,89 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:P2"/>
+  <sheetFormatPr customHeight="1"/>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>Company Name</v>
-      </c>
-      <c r="B1" t="str">
-        <v>Plan Name</v>
-      </c>
-      <c r="C1" t="str">
-        <v>States Covered</v>
-      </c>
-      <c r="D1" t="str">
-        <v>Formulary URL</v>
-      </c>
-      <c r="E1" t="str">
-        <v>Contact Phone</v>
-      </c>
-      <c r="F1" t="str">
-        <v xml:space="preserve">Communication Address Line 1 </v>
-      </c>
-      <c r="G1" t="str">
-        <v>Communication Address Line 2</v>
-      </c>
-      <c r="H1" t="str">
-        <v>City</v>
-      </c>
-      <c r="I1" t="str">
-        <v>State</v>
-      </c>
-      <c r="J1" t="str">
-        <v>Zip</v>
-      </c>
-      <c r="K1" t="str">
-        <v>Formulory date</v>
-      </c>
-      <c r="L1" t="str">
-        <v>Captured Date</v>
-      </c>
-      <c r="M1" t="str">
-        <v>Source Link</v>
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" t="s">
+        <v>12</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>Hennepin Health</v>
-      </c>
-      <c r="B2" t="str">
-        <v>Hennepin Health-MNCare</v>
-      </c>
-      <c r="C2" t="str">
-        <v/>
-      </c>
-      <c r="D2" t="str">
-        <v>https://www.iowamedicaidpdl.com/content/dam/ffs-medicare/ia/iowa-webpdl-100125.pdf</v>
-      </c>
-      <c r="E2" t="str">
-        <v>1-612-596-1036 (TTY 711)</v>
-      </c>
-      <c r="F2" t="str">
-        <v>300 South Sixth Street, MC 604</v>
-      </c>
-      <c r="G2" t="str">
-        <v/>
-      </c>
-      <c r="H2" t="str">
-        <v>Minneapolis</v>
-      </c>
-      <c r="I2" t="str">
-        <v xml:space="preserve"> Minnesota</v>
-      </c>
-      <c r="J2" t="str">
-        <v>55487-0604</v>
-      </c>
-      <c r="K2" t="str">
-        <v>11/1/2025</v>
-      </c>
-      <c r="L2" t="str">
-        <v>11/14/2025</v>
-      </c>
-      <c r="M2" t="str">
-        <v/>
-      </c>
-      <c r="N2" t="str">
-        <v>https://www.hennepinhealth.org/</v>
-      </c>
-      <c r="O2" t="str">
-        <v/>
-      </c>
-      <c r="P2" t="str">
-        <v>Madhan</v>
+    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E2" t="s">
+        <v>16</v>
+      </c>
+      <c r="F2" t="s">
+        <v>17</v>
+      </c>
+      <c r="H2" t="s">
+        <v>18</v>
+      </c>
+      <c r="I2" t="s">
+        <v>19</v>
+      </c>
+      <c r="J2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K2" t="s">
+        <v>21</v>
+      </c>
+      <c r="L2" t="s">
+        <v>22</v>
+      </c>
+      <c r="N2" t="s">
+        <v>23</v>
+      </c>
+      <c r="P2" t="s">
+        <v>24</v>
       </c>
     </row>
   </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:P2"/>
-  </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
few code changes as per the blockers
</commit_message>
<xml_diff>
--- a/errors.xlsx
+++ b/errors.xlsx
@@ -1,104 +1,47 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet sheetId="1" name="Sheet1" state="visible" r:id="rId4"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="171027"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
-  <si>
-    <t>Company Name</t>
-  </si>
-  <si>
-    <t>Plan Name</t>
-  </si>
-  <si>
-    <t>States Covered</t>
-  </si>
-  <si>
-    <t>Formulary URL</t>
-  </si>
-  <si>
-    <t>Contact Phone</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Communication Address Line 1 </t>
-  </si>
-  <si>
-    <t>Communication Address Line 2</t>
-  </si>
-  <si>
-    <t>City</t>
-  </si>
-  <si>
-    <t>State</t>
-  </si>
-  <si>
-    <t>Zip</t>
-  </si>
-  <si>
-    <t>Formulory date</t>
-  </si>
-  <si>
-    <t>Captured Date</t>
-  </si>
-  <si>
-    <t>Source Link</t>
-  </si>
-  <si>
-    <t>Hennepin Health</t>
-  </si>
-  <si>
-    <t>Hennepin Health-MNCare</t>
-  </si>
-  <si>
-    <t>https://cbg.adaptiverx.com/web/pdf?key=8F02B26A288102C27BAC82D14C006C6FC54D480F80409B6872E9A8AAA274F8DE</t>
-  </si>
-  <si>
-    <t>1-612-596-1036 (TTY 711)</t>
-  </si>
-  <si>
-    <t>300 South Sixth Street, MC 604</t>
-  </si>
-  <si>
-    <t>Minneapolis</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Minnesota</t>
-  </si>
-  <si>
-    <t>55487-0604</t>
-  </si>
-  <si>
-    <t>11/1/2025</t>
-  </si>
-  <si>
-    <t>11/14/2025</t>
-  </si>
-  <si>
-    <t>https://www.hennepinhealth.org/</t>
-  </si>
-  <si>
-    <t>Madhan</t>
-  </si>
-</sst>
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
+  <numFmts count="1">
+    <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
+  </numFmts>
+  <fonts count="1">
     <font>
+      <sz val="12"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="2">
@@ -122,21 +65,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
 </styleSheet>
 </file>
 
@@ -461,89 +396,91 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:P2"/>
-  <sheetFormatPr customHeight="1"/>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" t="s">
-        <v>8</v>
-      </c>
-      <c r="J1" t="s">
-        <v>9</v>
-      </c>
-      <c r="K1" t="s">
-        <v>10</v>
-      </c>
-      <c r="L1" t="s">
-        <v>11</v>
-      </c>
-      <c r="M1" t="s">
-        <v>12</v>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Company Name</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Plan Name</v>
+      </c>
+      <c r="C1" t="str">
+        <v>States Covered</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Formulary URL</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Contact Phone</v>
+      </c>
+      <c r="F1" t="str">
+        <v xml:space="preserve">Communication Address Line 1 </v>
+      </c>
+      <c r="G1" t="str">
+        <v>Communication Address Line 2</v>
+      </c>
+      <c r="H1" t="str">
+        <v>City</v>
+      </c>
+      <c r="I1" t="str">
+        <v>State</v>
+      </c>
+      <c r="J1" t="str">
+        <v>Zip</v>
+      </c>
+      <c r="K1" t="str">
+        <v>Formulory date</v>
+      </c>
+      <c r="L1" t="str">
+        <v>Captured Date</v>
+      </c>
+      <c r="M1" t="str">
+        <v>Source Link</v>
       </c>
     </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>13</v>
-      </c>
-      <c r="B2" t="s">
-        <v>14</v>
-      </c>
-      <c r="D2" t="s">
-        <v>15</v>
-      </c>
-      <c r="E2" t="s">
-        <v>16</v>
-      </c>
-      <c r="F2" t="s">
-        <v>17</v>
-      </c>
-      <c r="H2" t="s">
-        <v>18</v>
-      </c>
-      <c r="I2" t="s">
-        <v>19</v>
-      </c>
-      <c r="J2" t="s">
-        <v>20</v>
-      </c>
-      <c r="K2" t="s">
-        <v>21</v>
-      </c>
-      <c r="L2" t="s">
-        <v>22</v>
-      </c>
-      <c r="N2" t="s">
-        <v>23</v>
-      </c>
-      <c r="P2" t="s">
-        <v>24</v>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Hennepin Health</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Hennepin Health-MNCare</v>
+      </c>
+      <c r="D2" t="str">
+        <v>https://www.healthpartnersplans.com/content/dam/jeffersonhealthplans/documents/formularies/ifp/rxflex-formulary-jhp-ifp-2025-10012025.pdf</v>
+      </c>
+      <c r="E2" t="str">
+        <v>1-612-596-1036 (TTY 711)</v>
+      </c>
+      <c r="F2" t="str">
+        <v>300 South Sixth Street, MC 604</v>
+      </c>
+      <c r="H2" t="str">
+        <v>Minneapolis</v>
+      </c>
+      <c r="I2" t="str">
+        <v xml:space="preserve"> Minnesota</v>
+      </c>
+      <c r="J2" t="str">
+        <v>55487-0604</v>
+      </c>
+      <c r="K2" t="str">
+        <v>11/1/2025</v>
+      </c>
+      <c r="L2" t="str">
+        <v>11/14/2025</v>
+      </c>
+      <c r="N2" t="str">
+        <v>https://www.hennepinhealth.org/</v>
+      </c>
+      <c r="P2" t="str">
+        <v>Madhan</v>
       </c>
     </row>
   </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:P2"/>
+  </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
my code with prefreed agents template
</commit_message>
<xml_diff>
--- a/errors.xlsx
+++ b/errors.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P2"/>
+  <dimension ref="A1:M2"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -442,45 +442,48 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Hennepin Health</v>
+        <v>Priority Health</v>
       </c>
       <c r="B2" t="str">
-        <v>Hennepin Health-MNCare</v>
+        <v>(Individual/Family-MyPriority Plans</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Michigan</v>
       </c>
       <c r="D2" t="str">
-        <v>https://www.healthpartnersplans.com/content/dam/jeffersonhealthplans/documents/formularies/ifp/rxflex-formulary-jhp-ifp-2025-10012025.pdf</v>
+        <v>https://hcpf.colorado.gov/sites/hcpf/files/10-01-25%20PDL%20V3.pdf</v>
       </c>
       <c r="E2" t="str">
-        <v>1-612-596-1036 (TTY 711)</v>
+        <v>1-833-489-5443</v>
       </c>
       <c r="F2" t="str">
-        <v>300 South Sixth Street, MC 604</v>
+        <v>P.O. Box 232</v>
+      </c>
+      <c r="G2" t="str">
+        <v xml:space="preserve"> </v>
       </c>
       <c r="H2" t="str">
-        <v>Minneapolis</v>
+        <v>Grand Rapids</v>
       </c>
       <c r="I2" t="str">
-        <v xml:space="preserve"> Minnesota</v>
+        <v>Michigan</v>
       </c>
       <c r="J2" t="str">
-        <v>55487-0604</v>
+        <v>49501</v>
       </c>
       <c r="K2" t="str">
-        <v>11/1/2025</v>
+        <v>8-Dec-2025</v>
       </c>
       <c r="L2" t="str">
-        <v>11/14/2025</v>
-      </c>
-      <c r="N2" t="str">
-        <v>https://www.hennepinhealth.org/</v>
-      </c>
-      <c r="P2" t="str">
-        <v>Madhan</v>
+        <v>11-Dec-2025</v>
+      </c>
+      <c r="M2" t="str">
+        <v>https://www.priorityhealth.com/formulary/medical-drug-list/commercial-mypriority-current-year</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:P2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M2"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
solved index page issues and integrated prefreed agents template
</commit_message>
<xml_diff>
--- a/errors.xlsx
+++ b/errors.xlsx
@@ -442,16 +442,16 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Hennepin Health</v>
+        <v>Hennepin Health_12</v>
       </c>
       <c r="B2" t="str">
-        <v>Hennepin Health NCare</v>
+        <v>Hennepin Health NCare_1234</v>
       </c>
       <c r="C2" t="str">
         <v>Arkansas</v>
       </c>
       <c r="D2" t="str">
-        <v>https://www.securityhealth.org/-/media/Employers/2026-Employer-Document-Library/__2026_Sanford_Security_HIX_4T_Comprehensive_26215_v4_10232025.pdf?la=en&amp;hash=CB7C68A09BA95BA96DC94737E88AF6F4</v>
+        <v>https://www.kdhe.ks.gov/DocumentCenter/View/420/Preferred-Drug-List-PDF?bidId=</v>
       </c>
       <c r="E2" t="str">
         <v>1-612-596-1036 (TTY 711)</v>

</xml_diff>